<commit_message>
Sprint 17 Code Merged
</commit_message>
<xml_diff>
--- a/testcases/add-product-code/item-search-add-product-code.xlsx
+++ b/testcases/add-product-code/item-search-add-product-code.xlsx
@@ -52,7 +52,7 @@
     <t>Notes / Reason</t>
   </si>
   <si>
-    <t>TC-ISR-PCD-006</t>
+    <t>TC-ISR-PCD-001</t>
   </si>
   <si>
     <t>Add Product Code opens a required-empty form with Save held back</t>
@@ -111,193 +111,193 @@
     <t>Save is disabled</t>
   </si>
   <si>
+    <t>TC-ISR-PCD-002</t>
+  </si>
+  <si>
+    <t>Choosing a Product Type unlocks and filters Service Type</t>
+  </si>
+  <si>
+    <t>The Add Product Code dialog is open (previous case state)</t>
+  </si>
+  <si>
+    <t>1. Open the Product Type selector</t>
+  </si>
+  <si>
+    <t>Ten types are offered, including EQUIPMENT, CONSUMABLE, LABOR and FEE</t>
+  </si>
+  <si>
+    <t>2. Choose LABOR</t>
+  </si>
+  <si>
+    <t>The Service Type selector unlocks</t>
+  </si>
+  <si>
+    <t>3. Open the Service Type selector</t>
+  </si>
+  <si>
+    <t>Only labor services are offered (a list including Operator Labor, Rigging Labor and Setup Charges)</t>
+  </si>
+  <si>
+    <t>4. Press Escape, then close the dialog</t>
+  </si>
+  <si>
+    <t>The dialog closes; nothing is saved</t>
+  </si>
+  <si>
+    <t>TC-ISR-PCD-003</t>
+  </si>
+  <si>
+    <t>The Add segment menu opens per-segment forms</t>
+  </si>
+  <si>
+    <t>A result row is selected; no dialog open</t>
+  </si>
+  <si>
+    <t>1. Click the arrow beside Add Product Code</t>
+  </si>
+  <si>
+    <t>A menu lists Item, Sub Class, Class, Sub Category, Category</t>
+  </si>
+  <si>
+    <t>2. Click Category</t>
+  </si>
+  <si>
+    <t>The dialog opens and its single tab is named "Category"</t>
+  </si>
+  <si>
+    <t>3. Close the dialog</t>
+  </si>
+  <si>
+    <t>The grid is unchanged</t>
+  </si>
+  <si>
+    <t>TC-ISR-PCD-004</t>
+  </si>
+  <si>
+    <t>A completed Add Product Code form saves and the new code is found again</t>
+  </si>
+  <si>
+    <t>A default search has been executed on the Products page for office 1101 and a result row is selected (the new code is created under that row's category hierarchy)</t>
+  </si>
+  <si>
+    <t>1. Open Add Product Code and fill Name and Item Description with a per-run unique value (e.g. a ZZ-E2E-&lt;timestamp&gt; name)</t>
+  </si>
+  <si>
+    <t>Both required text fields hold the typed values, read back from the boxes</t>
+  </si>
+  <si>
+    <t>2. Choose Product Type EQUIPMENT, then choose Service Type Equipment Rental</t>
+  </si>
+  <si>
+    <t>Service Type unlocks once the Product Type is set; with all four required fields present, Save enables</t>
+  </si>
+  <si>
+    <t>3. Click Save</t>
+  </si>
+  <si>
+    <t>A "Product created successfully." toast appears and the dialog closes; `POST /navigator/api/product/create` returns success with a new id</t>
+  </si>
+  <si>
+    <t>4. Reset the search, type the new code's exact Name into Any Field, and click Search</t>
+  </si>
+  <si>
+    <t>Exactly one row returns — the product just created, carrying the category path of the row that was selected when Add opened</t>
+  </si>
+  <si>
+    <t>TC-ISR-PCD-005</t>
+  </si>
+  <si>
+    <t>The text fields stop accepting input at their maximum lengths</t>
+  </si>
+  <si>
+    <t>A search has been run on the Products page for office 1101, a result row is selected, and the Add Product Code dialog is open on the Item segment</t>
+  </si>
+  <si>
+    <t>1. Type 60 characters into Name</t>
+  </si>
+  <si>
+    <t>Exactly 50 characters land in the box; the extra 10 are never accepted</t>
+  </si>
+  <si>
+    <t>2. Read the Name box's error state</t>
+  </si>
+  <si>
+    <t>The field is not flagged invalid and no error message is shown — the field simply stopped accepting input</t>
+  </si>
+  <si>
+    <t>3. Type 70 characters into Item Description</t>
+  </si>
+  <si>
+    <t>Exactly 50 characters land in the box, with no error message</t>
+  </si>
+  <si>
+    <t>4. Type 15 digits into Oracle Item Number</t>
+  </si>
+  <si>
+    <t>Exactly 10 characters land in the box</t>
+  </si>
+  <si>
+    <t>TC-ISR-PCD-006</t>
+  </si>
+  <si>
+    <t>An over-length value that bypasses the typing limit cannot be saved</t>
+  </si>
+  <si>
+    <t>A result row is selected and the Add Product Code dialog is open on the Item segment</t>
+  </si>
+  <si>
+    <t>1. Put a 60-character value into Name and into Item Description by a route that bypasses the typing limit (the paste/scripted-fill path)</t>
+  </si>
+  <si>
+    <t>Both boxes hold all 60 characters — the typing limit does not apply to this route</t>
+  </si>
+  <si>
+    <t>2. Choose Product Type LABOR, then Service Type Application Development</t>
+  </si>
+  <si>
+    <t>Service Type unlocks and accepts the choice, so every required field now holds a value</t>
+  </si>
+  <si>
+    <t>3. Read the two text fields' error state and the Save button</t>
+  </si>
+  <si>
+    <t>Both fields are flagged invalid and Save is disabled, even though all four required fields are filled</t>
+  </si>
+  <si>
+    <t>4. Replace both values with valid short ones by the same route</t>
+  </si>
+  <si>
+    <t>Both fields clear their invalid flag and Save becomes enabled</t>
+  </si>
+  <si>
     <t>TC-ISR-PCD-007</t>
   </si>
   <si>
-    <t>Choosing a Product Type unlocks and filters Service Type</t>
-  </si>
-  <si>
-    <t>The Add Product Code dialog is open (previous case state)</t>
-  </si>
-  <si>
-    <t>1. Open the Product Type selector</t>
-  </si>
-  <si>
-    <t>Ten types are offered, including EQUIPMENT, CONSUMABLE, LABOR and FEE</t>
-  </si>
-  <si>
-    <t>2. Choose LABOR</t>
-  </si>
-  <si>
-    <t>The Service Type selector unlocks</t>
-  </si>
-  <si>
-    <t>3. Open the Service Type selector</t>
-  </si>
-  <si>
-    <t>Only labor services are offered (a list including Operator Labor, Rigging Labor and Setup Charges)</t>
-  </si>
-  <si>
-    <t>4. Press Escape, then close the dialog</t>
-  </si>
-  <si>
-    <t>The dialog closes; nothing is saved</t>
+    <t>A name at exactly the maximum length saves and reads back complete</t>
+  </si>
+  <si>
+    <t>1. Open Add Product Code and fill Name with a per-run unique value that is exactly 50 characters long, plus an Item Description</t>
+  </si>
+  <si>
+    <t>The Name box holds all 50 characters, read back from the box</t>
+  </si>
+  <si>
+    <t>2. Choose Product Type EQUIPMENT, then Service Type Equipment Rental</t>
+  </si>
+  <si>
+    <t>Save enables</t>
+  </si>
+  <si>
+    <t>A "Product created successfully." toast appears and the dialog closes; the create call returns success</t>
+  </si>
+  <si>
+    <t>4. Reset the search, type the full 50-character name into Any Field and search</t>
+  </si>
+  <si>
+    <t>Exactly one row returns and its Item cell holds all 50 characters — the value was stored whole, not shortened</t>
   </si>
   <si>
     <t>TC-ISR-PCD-008</t>
-  </si>
-  <si>
-    <t>The Add segment menu opens per-segment forms</t>
-  </si>
-  <si>
-    <t>A result row is selected; no dialog open</t>
-  </si>
-  <si>
-    <t>1. Click the arrow beside Add Product Code</t>
-  </si>
-  <si>
-    <t>A menu lists Item, Sub Class, Class, Sub Category, Category</t>
-  </si>
-  <si>
-    <t>2. Click Category</t>
-  </si>
-  <si>
-    <t>The dialog opens and its single tab is named "Category"</t>
-  </si>
-  <si>
-    <t>3. Close the dialog</t>
-  </si>
-  <si>
-    <t>The grid is unchanged</t>
-  </si>
-  <si>
-    <t>TC-ISR-PCD-011</t>
-  </si>
-  <si>
-    <t>A completed Add Product Code form saves and the new code is found again</t>
-  </si>
-  <si>
-    <t>A default search has been executed on the Products page for office 1101 and a result row is selected (the new code is created under that row's category hierarchy)</t>
-  </si>
-  <si>
-    <t>1. Open Add Product Code and fill Name and Item Description with a per-run unique value (e.g. a ZZ-E2E-&lt;timestamp&gt; name)</t>
-  </si>
-  <si>
-    <t>Both required text fields hold the typed values, read back from the boxes</t>
-  </si>
-  <si>
-    <t>2. Choose Product Type EQUIPMENT, then choose Service Type Equipment Rental</t>
-  </si>
-  <si>
-    <t>Service Type unlocks once the Product Type is set; with all four required fields present, Save enables</t>
-  </si>
-  <si>
-    <t>3. Click Save</t>
-  </si>
-  <si>
-    <t>A "Product created successfully." toast appears and the dialog closes; `POST /navigator/api/product/create` returns success with a new id</t>
-  </si>
-  <si>
-    <t>4. Reset the search, type the new code's exact Name into Any Field, and click Search</t>
-  </si>
-  <si>
-    <t>Exactly one row returns — the product just created, carrying the category path of the row that was selected when Add opened</t>
-  </si>
-  <si>
-    <t>TC-ISR-PCD-012</t>
-  </si>
-  <si>
-    <t>The text fields stop accepting input at their maximum lengths</t>
-  </si>
-  <si>
-    <t>A search has been run on the Products page for office 1101, a result row is selected, and the Add Product Code dialog is open on the Item segment</t>
-  </si>
-  <si>
-    <t>1. Type 60 characters into Name</t>
-  </si>
-  <si>
-    <t>Exactly 50 characters land in the box; the extra 10 are never accepted</t>
-  </si>
-  <si>
-    <t>2. Read the Name box's error state</t>
-  </si>
-  <si>
-    <t>The field is not flagged invalid and no error message is shown — the field simply stopped accepting input</t>
-  </si>
-  <si>
-    <t>3. Type 70 characters into Item Description</t>
-  </si>
-  <si>
-    <t>Exactly 50 characters land in the box, with no error message</t>
-  </si>
-  <si>
-    <t>4. Type 15 digits into Oracle Item Number</t>
-  </si>
-  <si>
-    <t>Exactly 10 characters land in the box</t>
-  </si>
-  <si>
-    <t>TC-ISR-PCD-013</t>
-  </si>
-  <si>
-    <t>An over-length value that bypasses the typing limit cannot be saved</t>
-  </si>
-  <si>
-    <t>A result row is selected and the Add Product Code dialog is open on the Item segment</t>
-  </si>
-  <si>
-    <t>1. Put a 60-character value into Name and into Item Description by a route that bypasses the typing limit (the paste/scripted-fill path)</t>
-  </si>
-  <si>
-    <t>Both boxes hold all 60 characters — the typing limit does not apply to this route</t>
-  </si>
-  <si>
-    <t>2. Choose Product Type LABOR, then Service Type Application Development</t>
-  </si>
-  <si>
-    <t>Service Type unlocks and accepts the choice, so every required field now holds a value</t>
-  </si>
-  <si>
-    <t>3. Read the two text fields' error state and the Save button</t>
-  </si>
-  <si>
-    <t>Both fields are flagged invalid and Save is disabled, even though all four required fields are filled</t>
-  </si>
-  <si>
-    <t>4. Replace both values with valid short ones by the same route</t>
-  </si>
-  <si>
-    <t>Both fields clear their invalid flag and Save becomes enabled</t>
-  </si>
-  <si>
-    <t>TC-ISR-PCD-014</t>
-  </si>
-  <si>
-    <t>A name at exactly the 50-character limit saves and reads back complete</t>
-  </si>
-  <si>
-    <t>1. Open Add Product Code and fill Name with a per-run unique value that is exactly 50 characters long, plus an Item Description</t>
-  </si>
-  <si>
-    <t>The Name box holds all 50 characters, read back from the box</t>
-  </si>
-  <si>
-    <t>2. Choose Product Type EQUIPMENT, then Service Type Equipment Rental</t>
-  </si>
-  <si>
-    <t>Save enables</t>
-  </si>
-  <si>
-    <t>A "Product created successfully." toast appears and the dialog closes; the create call returns success</t>
-  </si>
-  <si>
-    <t>4. Reset the search, type the full 50-character name into Any Field and search</t>
-  </si>
-  <si>
-    <t>Exactly one row returns and its Item cell holds all 50 characters — the value was stored whole, not shortened</t>
-  </si>
-  <si>
-    <t>TC-ISR-PCD-015</t>
   </si>
   <si>
     <t>Closing the Add dialog with a part-filled form discards it silently</t>

</xml_diff>

<commit_message>
Encore deliverable — NM-2255, NM-2258 and NM-2259 merged onto NM-3834 (14bb666)
</commit_message>
<xml_diff>
--- a/testcases/add-product-code/item-search-add-product-code.xlsx
+++ b/testcases/add-product-code/item-search-add-product-code.xlsx
@@ -52,7 +52,7 @@
     <t>Notes / Reason</t>
   </si>
   <si>
-    <t>TC-ISR-PCD-001</t>
+    <t>TC-ISR-APC-001</t>
   </si>
   <si>
     <t>Add Product Code opens a required-empty form with Save held back</t>
@@ -111,7 +111,7 @@
     <t>Save is disabled</t>
   </si>
   <si>
-    <t>TC-ISR-PCD-002</t>
+    <t>TC-ISR-APC-002</t>
   </si>
   <si>
     <t>Choosing a Product Type unlocks and filters Service Type</t>
@@ -144,7 +144,7 @@
     <t>The dialog closes; nothing is saved</t>
   </si>
   <si>
-    <t>TC-ISR-PCD-003</t>
+    <t>TC-ISR-APC-003</t>
   </si>
   <si>
     <t>The Add segment menu opens per-segment forms</t>
@@ -171,7 +171,7 @@
     <t>The grid is unchanged</t>
   </si>
   <si>
-    <t>TC-ISR-PCD-004</t>
+    <t>TC-ISR-APC-004</t>
   </si>
   <si>
     <t>A completed Add Product Code form saves and the new code is found again</t>
@@ -204,7 +204,7 @@
     <t>Exactly one row returns — the product just created, carrying the category path of the row that was selected when Add opened</t>
   </si>
   <si>
-    <t>TC-ISR-PCD-005</t>
+    <t>TC-ISR-APC-005</t>
   </si>
   <si>
     <t>The text fields stop accepting input at their maximum lengths</t>
@@ -237,7 +237,7 @@
     <t>Exactly 10 characters land in the box</t>
   </si>
   <si>
-    <t>TC-ISR-PCD-006</t>
+    <t>TC-ISR-APC-006</t>
   </si>
   <si>
     <t>An over-length value that bypasses the typing limit cannot be saved</t>
@@ -270,10 +270,10 @@
     <t>Both fields clear their invalid flag and Save becomes enabled</t>
   </si>
   <si>
-    <t>TC-ISR-PCD-007</t>
-  </si>
-  <si>
-    <t>A name at exactly the maximum length saves and reads back complete</t>
+    <t>TC-ISR-APC-007</t>
+  </si>
+  <si>
+    <t>A name at exactly the 50-character limit saves and reads back complete</t>
   </si>
   <si>
     <t>1. Open Add Product Code and fill Name with a per-run unique value that is exactly 50 characters long, plus an Item Description</t>
@@ -297,7 +297,7 @@
     <t>Exactly one row returns and its Item cell holds all 50 characters — the value was stored whole, not shortened</t>
   </si>
   <si>
-    <t>TC-ISR-PCD-008</t>
+    <t>TC-ISR-APC-008</t>
   </si>
   <si>
     <t>Closing the Add dialog with a part-filled form discards it silently</t>
@@ -342,7 +342,7 @@
     <t>Pass:8 Fail:0 Skipped:0 Blocked:0</t>
   </si>
   <si>
-    <t>Last Updated: 2026-09-04</t>
+    <t>Last Updated: 2026-09-16</t>
   </si>
 </sst>
 </file>

</xml_diff>